<commit_message>
Enhance app to test hypothesis: Does Higher Budget Lower Crime Rate with 4-Quadrant Matrix
</commit_message>
<xml_diff>
--- a/crime_data.xlsx
+++ b/crime_data.xlsx
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13996419239</v>
+        <v>14811833563</v>
       </c>
       <c r="C2" t="n">
         <v>10181</v>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9838715103</v>
+        <v>14359866175</v>
       </c>
       <c r="C3" t="n">
         <v>10142</v>
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18097722907</v>
+        <v>10345695687</v>
       </c>
       <c r="C4" t="n">
         <v>10276</v>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11667177512</v>
+        <v>14934502256</v>
       </c>
       <c r="C5" t="n">
         <v>8427</v>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18386241172</v>
+        <v>21714063705</v>
       </c>
       <c r="C6" t="n">
         <v>10401</v>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24758068702</v>
+        <v>14450932137</v>
       </c>
       <c r="C7" t="n">
         <v>11196</v>
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25316427638</v>
+        <v>24613526943</v>
       </c>
       <c r="C8" t="n">
         <v>10403</v>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24354994795</v>
+        <v>21615494869</v>
       </c>
       <c r="C9" t="n">
         <v>9045</v>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21110637956</v>
+        <v>16069000634</v>
       </c>
       <c r="C10" t="n">
         <v>8786</v>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13688284923</v>
+        <v>17247482181</v>
       </c>
       <c r="C11" t="n">
         <v>6939</v>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>35657240433</v>
+        <v>30517059143</v>
       </c>
       <c r="C12" t="n">
         <v>9981</v>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>24043191129</v>
+        <v>27983132434</v>
       </c>
       <c r="C13" t="n">
         <v>10293</v>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19528834476</v>
+        <v>21379023145</v>
       </c>
       <c r="C14" t="n">
         <v>7322</v>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>19025095867</v>
+        <v>15842528047</v>
       </c>
       <c r="C15" t="n">
         <v>14406</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15443647333</v>
+        <v>20310331826</v>
       </c>
       <c r="C16" t="n">
         <v>10332</v>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>23293221081</v>
+        <v>35956011833</v>
       </c>
       <c r="C17" t="n">
         <v>15664</v>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>15907442565</v>
+        <v>15609441447</v>
       </c>
       <c r="C18" t="n">
         <v>12342</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>15759120158</v>
+        <v>18641035217</v>
       </c>
       <c r="C19" t="n">
         <v>8730</v>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>21077997436</v>
+        <v>14785792420</v>
       </c>
       <c r="C20" t="n">
         <v>15764</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>17598868606</v>
+        <v>26923234514</v>
       </c>
       <c r="C22" t="n">
         <v>16391</v>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>14393636080</v>
+        <v>22488566111</v>
       </c>
       <c r="C23" t="n">
         <v>17536</v>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>35294135421</v>
+        <v>21251196973</v>
       </c>
       <c r="C24" t="n">
         <v>33190</v>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>31856552551</v>
+        <v>32411658313</v>
       </c>
       <c r="C25" t="n">
         <v>19498</v>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>17569662193</v>
+        <v>21602707031</v>
       </c>
       <c r="C26" t="n">
         <v>12097</v>

</xml_diff>

<commit_message>
Implement map-centric UI with permanently visible labels on Leaflet map
</commit_message>
<xml_diff>
--- a/crime_data.xlsx
+++ b/crime_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G230"/>
+  <dimension ref="A1:I230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,16 @@
           <t>특이사항</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>위도</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>경도</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -493,6 +503,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H2" t="n">
+        <v>37.573</v>
+      </c>
+      <c r="I2" t="n">
+        <v>126.9794</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -522,6 +538,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>37.5636</v>
+      </c>
+      <c r="I3" t="n">
+        <v>126.9975</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -551,6 +573,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>37.5326</v>
+      </c>
+      <c r="I4" t="n">
+        <v>126.99</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -580,6 +608,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>37.5633</v>
+      </c>
+      <c r="I5" t="n">
+        <v>127.0371</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -609,6 +643,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H6" t="n">
+        <v>37.5385</v>
+      </c>
+      <c r="I6" t="n">
+        <v>127.0822</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -638,6 +678,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H7" t="n">
+        <v>37.5744</v>
+      </c>
+      <c r="I7" t="n">
+        <v>127.04</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -667,6 +713,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H8" t="n">
+        <v>37.6065</v>
+      </c>
+      <c r="I8" t="n">
+        <v>127.0927</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -696,6 +748,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H9" t="n">
+        <v>37.5891</v>
+      </c>
+      <c r="I9" t="n">
+        <v>127.0182</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -725,6 +783,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H10" t="n">
+        <v>37.6396</v>
+      </c>
+      <c r="I10" t="n">
+        <v>127.0257</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -754,6 +818,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H11" t="n">
+        <v>37.6688</v>
+      </c>
+      <c r="I11" t="n">
+        <v>127.0471</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -783,6 +853,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H12" t="n">
+        <v>37.6542</v>
+      </c>
+      <c r="I12" t="n">
+        <v>127.0568</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -812,6 +888,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H13" t="n">
+        <v>37.6027</v>
+      </c>
+      <c r="I13" t="n">
+        <v>126.9291</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -841,6 +923,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H14" t="n">
+        <v>37.5791</v>
+      </c>
+      <c r="I14" t="n">
+        <v>126.9368</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -870,6 +958,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H15" t="n">
+        <v>37.5662</v>
+      </c>
+      <c r="I15" t="n">
+        <v>126.9016</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -899,6 +993,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H16" t="n">
+        <v>37.5169</v>
+      </c>
+      <c r="I16" t="n">
+        <v>126.866</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -928,6 +1028,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H17" t="n">
+        <v>37.5509</v>
+      </c>
+      <c r="I17" t="n">
+        <v>126.8497</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -957,6 +1063,12 @@
           <t>산업단지 및 다문화/공업 밀집</t>
         </is>
       </c>
+      <c r="H18" t="n">
+        <v>37.4954</v>
+      </c>
+      <c r="I18" t="n">
+        <v>126.8874</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -986,6 +1098,12 @@
           <t>산업단지 및 다문화/공업 밀집</t>
         </is>
       </c>
+      <c r="H19" t="n">
+        <v>37.4568</v>
+      </c>
+      <c r="I19" t="n">
+        <v>126.8954</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1015,6 +1133,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H20" t="n">
+        <v>37.5264</v>
+      </c>
+      <c r="I20" t="n">
+        <v>126.8962</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1044,6 +1168,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H21" t="n">
+        <v>37.5124</v>
+      </c>
+      <c r="I21" t="n">
+        <v>126.9393</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1073,6 +1203,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H22" t="n">
+        <v>37.4784</v>
+      </c>
+      <c r="I22" t="n">
+        <v>126.9516</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1102,6 +1238,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H23" t="n">
+        <v>37.4837</v>
+      </c>
+      <c r="I23" t="n">
+        <v>127.0324</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1131,6 +1273,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H24" t="n">
+        <v>37.5172</v>
+      </c>
+      <c r="I24" t="n">
+        <v>127.0473</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1160,6 +1308,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H25" t="n">
+        <v>37.5145</v>
+      </c>
+      <c r="I25" t="n">
+        <v>127.1066</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1189,6 +1343,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H26" t="n">
+        <v>37.5301</v>
+      </c>
+      <c r="I26" t="n">
+        <v>127.1238</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1218,6 +1378,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H27" t="n">
+        <v>35.1062</v>
+      </c>
+      <c r="I27" t="n">
+        <v>129.0324</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1247,6 +1413,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H28" t="n">
+        <v>35.0979</v>
+      </c>
+      <c r="I28" t="n">
+        <v>129.0244</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1276,6 +1448,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H29" t="n">
+        <v>35.1293</v>
+      </c>
+      <c r="I29" t="n">
+        <v>129.0454</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1305,6 +1483,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H30" t="n">
+        <v>35.0912</v>
+      </c>
+      <c r="I30" t="n">
+        <v>129.0679</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1334,6 +1518,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H31" t="n">
+        <v>35.0746</v>
+      </c>
+      <c r="I31" t="n">
+        <v>128.7156</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1363,6 +1553,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H32" t="n">
+        <v>35.2048</v>
+      </c>
+      <c r="I32" t="n">
+        <v>129.0836</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1392,6 +1588,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H33" t="n">
+        <v>35.1365</v>
+      </c>
+      <c r="I33" t="n">
+        <v>129.0842</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1421,6 +1623,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H34" t="n">
+        <v>35.1972</v>
+      </c>
+      <c r="I34" t="n">
+        <v>128.9902</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1450,6 +1658,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H35" t="n">
+        <v>35.2122</v>
+      </c>
+      <c r="I35" t="n">
+        <v>128.9806</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1479,6 +1693,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H36" t="n">
+        <v>35.1631</v>
+      </c>
+      <c r="I36" t="n">
+        <v>129.1636</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1508,6 +1728,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H37" t="n">
+        <v>35.1045</v>
+      </c>
+      <c r="I37" t="n">
+        <v>128.9748</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1537,6 +1763,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H38" t="n">
+        <v>35.243</v>
+      </c>
+      <c r="I38" t="n">
+        <v>129.0921</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1566,6 +1798,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H39" t="n">
+        <v>35.1765</v>
+      </c>
+      <c r="I39" t="n">
+        <v>129.0797</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1595,6 +1833,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H40" t="n">
+        <v>35.1456</v>
+      </c>
+      <c r="I40" t="n">
+        <v>129.1132</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1624,6 +1868,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H41" t="n">
+        <v>35.1526</v>
+      </c>
+      <c r="I41" t="n">
+        <v>128.9912</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1653,6 +1903,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H42" t="n">
+        <v>35.2445</v>
+      </c>
+      <c r="I42" t="n">
+        <v>129.2224</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1682,6 +1938,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H43" t="n">
+        <v>35.8694</v>
+      </c>
+      <c r="I43" t="n">
+        <v>128.6062</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1711,6 +1973,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H44" t="n">
+        <v>35.8866</v>
+      </c>
+      <c r="I44" t="n">
+        <v>128.6358</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1740,6 +2008,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H45" t="n">
+        <v>35.8719</v>
+      </c>
+      <c r="I45" t="n">
+        <v>128.5591</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1769,6 +2043,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H46" t="n">
+        <v>35.8459</v>
+      </c>
+      <c r="I46" t="n">
+        <v>128.5974</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1798,6 +2078,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H47" t="n">
+        <v>35.8857</v>
+      </c>
+      <c r="I47" t="n">
+        <v>128.5828</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1827,6 +2113,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H48" t="n">
+        <v>35.8583</v>
+      </c>
+      <c r="I48" t="n">
+        <v>128.6306</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1856,6 +2148,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H49" t="n">
+        <v>35.8298</v>
+      </c>
+      <c r="I49" t="n">
+        <v>128.5327</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1885,6 +2183,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H50" t="n">
+        <v>35.7746</v>
+      </c>
+      <c r="I50" t="n">
+        <v>128.4313</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1914,6 +2218,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H51" t="n">
+        <v>36.2428</v>
+      </c>
+      <c r="I51" t="n">
+        <v>128.5728</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1943,6 +2253,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H52" t="n">
+        <v>37.4738</v>
+      </c>
+      <c r="I52" t="n">
+        <v>126.6216</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1972,6 +2288,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H53" t="n">
+        <v>37.4738</v>
+      </c>
+      <c r="I53" t="n">
+        <v>126.6432</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2001,6 +2323,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H54" t="n">
+        <v>37.4636</v>
+      </c>
+      <c r="I54" t="n">
+        <v>126.6502</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2030,6 +2358,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H55" t="n">
+        <v>37.4101</v>
+      </c>
+      <c r="I55" t="n">
+        <v>126.6783</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2059,6 +2393,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H56" t="n">
+        <v>37.447</v>
+      </c>
+      <c r="I56" t="n">
+        <v>126.7314</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2088,6 +2428,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H57" t="n">
+        <v>37.507</v>
+      </c>
+      <c r="I57" t="n">
+        <v>126.7218</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2117,6 +2463,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H58" t="n">
+        <v>37.5374</v>
+      </c>
+      <c r="I58" t="n">
+        <v>126.7377</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2146,6 +2498,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H59" t="n">
+        <v>37.5454</v>
+      </c>
+      <c r="I59" t="n">
+        <v>126.676</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2175,6 +2533,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H60" t="n">
+        <v>37.7465</v>
+      </c>
+      <c r="I60" t="n">
+        <v>126.488</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2204,6 +2568,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H61" t="n">
+        <v>37.4465</v>
+      </c>
+      <c r="I61" t="n">
+        <v>126.6368</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2233,6 +2603,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H62" t="n">
+        <v>35.146</v>
+      </c>
+      <c r="I62" t="n">
+        <v>126.9232</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2262,6 +2638,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H63" t="n">
+        <v>35.152</v>
+      </c>
+      <c r="I63" t="n">
+        <v>126.8897</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2291,6 +2673,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H64" t="n">
+        <v>35.1329</v>
+      </c>
+      <c r="I64" t="n">
+        <v>126.9025</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2320,6 +2708,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H65" t="n">
+        <v>35.1741</v>
+      </c>
+      <c r="I65" t="n">
+        <v>126.9121</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2349,6 +2743,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H66" t="n">
+        <v>35.1396</v>
+      </c>
+      <c r="I66" t="n">
+        <v>126.7937</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2378,6 +2778,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H67" t="n">
+        <v>36.312</v>
+      </c>
+      <c r="I67" t="n">
+        <v>127.455</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2407,6 +2813,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H68" t="n">
+        <v>36.3259</v>
+      </c>
+      <c r="I68" t="n">
+        <v>127.4214</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2436,6 +2848,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H69" t="n">
+        <v>36.3553</v>
+      </c>
+      <c r="I69" t="n">
+        <v>127.3837</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2465,6 +2883,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H70" t="n">
+        <v>36.3623</v>
+      </c>
+      <c r="I70" t="n">
+        <v>127.3564</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2494,6 +2918,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H71" t="n">
+        <v>36.3467</v>
+      </c>
+      <c r="I71" t="n">
+        <v>127.4156</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2523,6 +2953,12 @@
           <t>중심 상업/유흥 번화가 및 유동인구 집중</t>
         </is>
       </c>
+      <c r="H72" t="n">
+        <v>35.5698</v>
+      </c>
+      <c r="I72" t="n">
+        <v>129.3328</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2552,6 +2988,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H73" t="n">
+        <v>35.5438</v>
+      </c>
+      <c r="I73" t="n">
+        <v>129.3301</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2581,6 +3023,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H74" t="n">
+        <v>35.5049</v>
+      </c>
+      <c r="I74" t="n">
+        <v>129.4167</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2610,6 +3058,12 @@
           <t>산업단지 및 다문화/공업 밀집</t>
         </is>
       </c>
+      <c r="H75" t="n">
+        <v>35.5828</v>
+      </c>
+      <c r="I75" t="n">
+        <v>129.3615</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2639,6 +3093,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H76" t="n">
+        <v>35.5398</v>
+      </c>
+      <c r="I76" t="n">
+        <v>129.2374</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2668,6 +3128,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H77" t="n">
+        <v>36.48</v>
+      </c>
+      <c r="I77" t="n">
+        <v>127.289</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2697,6 +3163,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H78" t="n">
+        <v>37.6584</v>
+      </c>
+      <c r="I78" t="n">
+        <v>126.832</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2726,6 +3198,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H79" t="n">
+        <v>37.4292</v>
+      </c>
+      <c r="I79" t="n">
+        <v>126.9877</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2755,6 +3233,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H80" t="n">
+        <v>37.4786</v>
+      </c>
+      <c r="I80" t="n">
+        <v>126.8646</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2784,6 +3268,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H81" t="n">
+        <v>37.4294</v>
+      </c>
+      <c r="I81" t="n">
+        <v>127.2551</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2813,6 +3303,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H82" t="n">
+        <v>37.5943</v>
+      </c>
+      <c r="I82" t="n">
+        <v>127.1296</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2842,6 +3338,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H83" t="n">
+        <v>37.3614</v>
+      </c>
+      <c r="I83" t="n">
+        <v>126.9352</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2871,6 +3373,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H84" t="n">
+        <v>37.6152</v>
+      </c>
+      <c r="I84" t="n">
+        <v>126.7157</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2900,6 +3408,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H85" t="n">
+        <v>37.636</v>
+      </c>
+      <c r="I85" t="n">
+        <v>127.2165</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2929,6 +3443,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H86" t="n">
+        <v>37.9036</v>
+      </c>
+      <c r="I86" t="n">
+        <v>127.0607</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2958,6 +3478,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H87" t="n">
+        <v>37.5034</v>
+      </c>
+      <c r="I87" t="n">
+        <v>126.766</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2987,6 +3513,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H88" t="n">
+        <v>37.4201</v>
+      </c>
+      <c r="I88" t="n">
+        <v>127.1265</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3016,6 +3548,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H89" t="n">
+        <v>37.2636</v>
+      </c>
+      <c r="I89" t="n">
+        <v>127.0286</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3045,6 +3583,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H90" t="n">
+        <v>37.3802</v>
+      </c>
+      <c r="I90" t="n">
+        <v>126.8029</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3074,6 +3618,12 @@
           <t>산업단지 및 다문화/공업 밀집</t>
         </is>
       </c>
+      <c r="H91" t="n">
+        <v>37.3219</v>
+      </c>
+      <c r="I91" t="n">
+        <v>126.8309</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3103,6 +3653,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H92" t="n">
+        <v>37.008</v>
+      </c>
+      <c r="I92" t="n">
+        <v>127.2798</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3132,6 +3688,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H93" t="n">
+        <v>37.3943</v>
+      </c>
+      <c r="I93" t="n">
+        <v>126.9568</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3161,6 +3723,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H94" t="n">
+        <v>37.7853</v>
+      </c>
+      <c r="I94" t="n">
+        <v>127.0458</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3190,6 +3758,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H95" t="n">
+        <v>37.2984</v>
+      </c>
+      <c r="I95" t="n">
+        <v>127.6371</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3219,6 +3793,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H96" t="n">
+        <v>37.1498</v>
+      </c>
+      <c r="I96" t="n">
+        <v>127.0772</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3248,6 +3828,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H97" t="n">
+        <v>37.2411</v>
+      </c>
+      <c r="I97" t="n">
+        <v>127.1776</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3277,6 +3863,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H98" t="n">
+        <v>37.3448</v>
+      </c>
+      <c r="I98" t="n">
+        <v>126.9682</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3306,6 +3898,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H99" t="n">
+        <v>37.7381</v>
+      </c>
+      <c r="I99" t="n">
+        <v>127.0337</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3335,6 +3933,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H100" t="n">
+        <v>37.2723</v>
+      </c>
+      <c r="I100" t="n">
+        <v>127.435</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3364,6 +3968,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H101" t="n">
+        <v>37.76</v>
+      </c>
+      <c r="I101" t="n">
+        <v>126.7799</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3393,6 +4003,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H102" t="n">
+        <v>36.9921</v>
+      </c>
+      <c r="I102" t="n">
+        <v>127.1129</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3422,6 +4038,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H103" t="n">
+        <v>37.8949</v>
+      </c>
+      <c r="I103" t="n">
+        <v>127.2003</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3451,6 +4073,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H104" t="n">
+        <v>37.5393</v>
+      </c>
+      <c r="I104" t="n">
+        <v>127.2148</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3480,6 +4108,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H105" t="n">
+        <v>37.1995</v>
+      </c>
+      <c r="I105" t="n">
+        <v>126.8315</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3509,6 +4143,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H106" t="n">
+        <v>38.0964</v>
+      </c>
+      <c r="I106" t="n">
+        <v>127.0747</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3538,6 +4178,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H107" t="n">
+        <v>37.8315</v>
+      </c>
+      <c r="I107" t="n">
+        <v>127.5097</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3567,6 +4213,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H108" t="n">
+        <v>37.4917</v>
+      </c>
+      <c r="I108" t="n">
+        <v>127.4876</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3596,6 +4248,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H109" t="n">
+        <v>37.7519</v>
+      </c>
+      <c r="I109" t="n">
+        <v>128.8761</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3625,6 +4283,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H110" t="n">
+        <v>37.5247</v>
+      </c>
+      <c r="I110" t="n">
+        <v>129.1143</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3654,6 +4318,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H111" t="n">
+        <v>37.4499</v>
+      </c>
+      <c r="I111" t="n">
+        <v>129.1652</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3683,6 +4353,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H112" t="n">
+        <v>38.207</v>
+      </c>
+      <c r="I112" t="n">
+        <v>128.5918</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3712,6 +4388,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H113" t="n">
+        <v>37.3422</v>
+      </c>
+      <c r="I113" t="n">
+        <v>127.9202</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3741,6 +4423,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H114" t="n">
+        <v>37.8813</v>
+      </c>
+      <c r="I114" t="n">
+        <v>127.7298</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3770,6 +4458,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H115" t="n">
+        <v>37.1641</v>
+      </c>
+      <c r="I115" t="n">
+        <v>128.9856</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3799,6 +4493,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H116" t="n">
+        <v>37.6972</v>
+      </c>
+      <c r="I116" t="n">
+        <v>127.8887</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3828,6 +4528,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H117" t="n">
+        <v>37.4918</v>
+      </c>
+      <c r="I117" t="n">
+        <v>127.985</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3857,6 +4563,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H118" t="n">
+        <v>37.1838</v>
+      </c>
+      <c r="I118" t="n">
+        <v>128.4619</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3886,6 +4598,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H119" t="n">
+        <v>37.3705</v>
+      </c>
+      <c r="I119" t="n">
+        <v>128.3902</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3915,6 +4633,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H120" t="n">
+        <v>37.3806</v>
+      </c>
+      <c r="I120" t="n">
+        <v>128.6608</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3944,6 +4668,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H121" t="n">
+        <v>38.1468</v>
+      </c>
+      <c r="I121" t="n">
+        <v>127.3134</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3973,6 +4703,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H122" t="n">
+        <v>38.1062</v>
+      </c>
+      <c r="I122" t="n">
+        <v>127.7082</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4002,6 +4738,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H123" t="n">
+        <v>38.1079</v>
+      </c>
+      <c r="I123" t="n">
+        <v>127.9897</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4031,6 +4773,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H124" t="n">
+        <v>38.0697</v>
+      </c>
+      <c r="I124" t="n">
+        <v>128.1704</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4060,6 +4808,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H125" t="n">
+        <v>38.3806</v>
+      </c>
+      <c r="I125" t="n">
+        <v>128.4678</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4089,6 +4843,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H126" t="n">
+        <v>38.0754</v>
+      </c>
+      <c r="I126" t="n">
+        <v>128.6189</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4118,6 +4878,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H127" t="n">
+        <v>36.7407</v>
+      </c>
+      <c r="I127" t="n">
+        <v>127.7162</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4147,6 +4913,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H128" t="n">
+        <v>36.6007</v>
+      </c>
+      <c r="I128" t="n">
+        <v>127.5812</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4176,6 +4948,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H129" t="n">
+        <v>36.2507</v>
+      </c>
+      <c r="I129" t="n">
+        <v>127.1312</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4205,6 +4983,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H130" t="n">
+        <v>36.4607</v>
+      </c>
+      <c r="I130" t="n">
+        <v>126.8162</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4234,6 +5018,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H131" t="n">
+        <v>36.7407</v>
+      </c>
+      <c r="I131" t="n">
+        <v>127.3562</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4263,6 +5053,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H132" t="n">
+        <v>36.2857</v>
+      </c>
+      <c r="I132" t="n">
+        <v>126.8612</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4292,6 +5088,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H133" t="n">
+        <v>36.9507</v>
+      </c>
+      <c r="I133" t="n">
+        <v>127.7612</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4321,6 +5123,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H134" t="n">
+        <v>36.7757</v>
+      </c>
+      <c r="I134" t="n">
+        <v>127.3562</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4350,6 +5158,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H135" t="n">
+        <v>37.1257</v>
+      </c>
+      <c r="I135" t="n">
+        <v>127.7162</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4379,6 +5193,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H136" t="n">
+        <v>36.4257</v>
+      </c>
+      <c r="I136" t="n">
+        <v>128.0312</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4408,6 +5228,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H137" t="n">
+        <v>36.9857</v>
+      </c>
+      <c r="I137" t="n">
+        <v>127.2212</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4437,6 +5263,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H138" t="n">
+        <v>36.7634</v>
+      </c>
+      <c r="I138" t="n">
+        <v>126.305</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4466,6 +5298,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H139" t="n">
+        <v>36.6584</v>
+      </c>
+      <c r="I139" t="n">
+        <v>127.07</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4495,6 +5333,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H140" t="n">
+        <v>36.1684</v>
+      </c>
+      <c r="I140" t="n">
+        <v>126.53</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4524,6 +5368,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H141" t="n">
+        <v>37.0084</v>
+      </c>
+      <c r="I141" t="n">
+        <v>126.35</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4553,6 +5403,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H142" t="n">
+        <v>36.4834</v>
+      </c>
+      <c r="I142" t="n">
+        <v>126.935</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4582,6 +5438,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H143" t="n">
+        <v>36.2734</v>
+      </c>
+      <c r="I143" t="n">
+        <v>126.44</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4611,6 +5473,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H144" t="n">
+        <v>36.7284</v>
+      </c>
+      <c r="I144" t="n">
+        <v>126.89</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4640,6 +5508,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H145" t="n">
+        <v>36.2384</v>
+      </c>
+      <c r="I145" t="n">
+        <v>126.845</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4669,6 +5543,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H146" t="n">
+        <v>35.9934</v>
+      </c>
+      <c r="I146" t="n">
+        <v>126.98</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4698,6 +5578,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H147" t="n">
+        <v>36.6584</v>
+      </c>
+      <c r="I147" t="n">
+        <v>126.62</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4727,6 +5613,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H148" t="n">
+        <v>36.3784</v>
+      </c>
+      <c r="I148" t="n">
+        <v>126.53</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4756,6 +5648,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H149" t="n">
+        <v>36.1334</v>
+      </c>
+      <c r="I149" t="n">
+        <v>126.935</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4785,6 +5683,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H150" t="n">
+        <v>36.6584</v>
+      </c>
+      <c r="I150" t="n">
+        <v>126.17</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4814,6 +5718,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H151" t="n">
+        <v>36.3084</v>
+      </c>
+      <c r="I151" t="n">
+        <v>126.125</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4843,6 +5753,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H152" t="n">
+        <v>36.0984</v>
+      </c>
+      <c r="I152" t="n">
+        <v>126.125</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4872,6 +5788,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H153" t="n">
+        <v>35.9975</v>
+      </c>
+      <c r="I153" t="n">
+        <v>127.423</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4901,6 +5823,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H154" t="n">
+        <v>35.6125</v>
+      </c>
+      <c r="I154" t="n">
+        <v>127.243</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4930,6 +5858,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H155" t="n">
+        <v>35.6825</v>
+      </c>
+      <c r="I155" t="n">
+        <v>126.478</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4959,6 +5893,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H156" t="n">
+        <v>35.7525</v>
+      </c>
+      <c r="I156" t="n">
+        <v>127.333</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4988,6 +5928,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H157" t="n">
+        <v>35.4375</v>
+      </c>
+      <c r="I157" t="n">
+        <v>127.738</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5017,6 +5963,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H158" t="n">
+        <v>36.1025</v>
+      </c>
+      <c r="I158" t="n">
+        <v>127.018</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5046,6 +5998,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H159" t="n">
+        <v>35.4375</v>
+      </c>
+      <c r="I159" t="n">
+        <v>126.523</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5075,6 +6033,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H160" t="n">
+        <v>35.9275</v>
+      </c>
+      <c r="I160" t="n">
+        <v>127.738</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5104,6 +6068,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H161" t="n">
+        <v>35.9625</v>
+      </c>
+      <c r="I161" t="n">
+        <v>127.693</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5133,6 +6103,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H162" t="n">
+        <v>35.3675</v>
+      </c>
+      <c r="I162" t="n">
+        <v>127.648</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5162,6 +6138,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H163" t="n">
+        <v>36.1375</v>
+      </c>
+      <c r="I163" t="n">
+        <v>127.423</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5191,6 +6173,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H164" t="n">
+        <v>35.6475</v>
+      </c>
+      <c r="I164" t="n">
+        <v>127.828</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5220,6 +6208,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H165" t="n">
+        <v>35.3675</v>
+      </c>
+      <c r="I165" t="n">
+        <v>127.063</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5249,6 +6243,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H166" t="n">
+        <v>35.2275</v>
+      </c>
+      <c r="I166" t="n">
+        <v>127.513</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5278,6 +6278,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H167" t="n">
+        <v>34.5879</v>
+      </c>
+      <c r="I167" t="n">
+        <v>127.081</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5307,6 +6313,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H168" t="n">
+        <v>34.8679</v>
+      </c>
+      <c r="I168" t="n">
+        <v>126.406</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5336,6 +6348,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H169" t="n">
+        <v>35.2179</v>
+      </c>
+      <c r="I169" t="n">
+        <v>127.531</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5365,6 +6383,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H170" t="n">
+        <v>35.2879</v>
+      </c>
+      <c r="I170" t="n">
+        <v>127.666</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5394,6 +6418,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H171" t="n">
+        <v>35.3579</v>
+      </c>
+      <c r="I171" t="n">
+        <v>126.316</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5423,6 +6453,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H172" t="n">
+        <v>34.5879</v>
+      </c>
+      <c r="I172" t="n">
+        <v>127.531</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5452,6 +6488,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H173" t="n">
+        <v>35.1129</v>
+      </c>
+      <c r="I173" t="n">
+        <v>127.171</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5481,6 +6523,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H174" t="n">
+        <v>34.5179</v>
+      </c>
+      <c r="I174" t="n">
+        <v>127.261</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5510,6 +6558,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H175" t="n">
+        <v>35.0079</v>
+      </c>
+      <c r="I175" t="n">
+        <v>127.216</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5539,6 +6593,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H176" t="n">
+        <v>35.3929</v>
+      </c>
+      <c r="I176" t="n">
+        <v>127.531</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5568,6 +6628,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H177" t="n">
+        <v>35.3229</v>
+      </c>
+      <c r="I177" t="n">
+        <v>127.216</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5597,6 +6663,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H178" t="n">
+        <v>34.7629</v>
+      </c>
+      <c r="I178" t="n">
+        <v>126.946</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5626,6 +6698,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H179" t="n">
+        <v>35.0429</v>
+      </c>
+      <c r="I179" t="n">
+        <v>126.856</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -5655,6 +6733,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H180" t="n">
+        <v>35.1479</v>
+      </c>
+      <c r="I180" t="n">
+        <v>127.486</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -5684,6 +6768,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H181" t="n">
+        <v>34.8329</v>
+      </c>
+      <c r="I181" t="n">
+        <v>126.901</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5713,6 +6803,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H182" t="n">
+        <v>34.4129</v>
+      </c>
+      <c r="I182" t="n">
+        <v>127.666</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -5742,6 +6838,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H183" t="n">
+        <v>34.5529</v>
+      </c>
+      <c r="I183" t="n">
+        <v>126.631</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5771,6 +6873,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H184" t="n">
+        <v>35.0079</v>
+      </c>
+      <c r="I184" t="n">
+        <v>126.856</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5800,6 +6908,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H185" t="n">
+        <v>34.3429</v>
+      </c>
+      <c r="I185" t="n">
+        <v>127.216</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -5829,6 +6943,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H186" t="n">
+        <v>35.2529</v>
+      </c>
+      <c r="I186" t="n">
+        <v>127.126</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -5858,6 +6978,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H187" t="n">
+        <v>34.7279</v>
+      </c>
+      <c r="I187" t="n">
+        <v>127.396</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -5887,6 +7013,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H188" t="n">
+        <v>35.2179</v>
+      </c>
+      <c r="I188" t="n">
+        <v>126.586</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -5916,6 +7048,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H189" t="n">
+        <v>36.191</v>
+      </c>
+      <c r="I189" t="n">
+        <v>129.1806</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -5945,6 +7083,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H190" t="n">
+        <v>36.156</v>
+      </c>
+      <c r="I190" t="n">
+        <v>128.2806</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -5974,6 +7118,12 @@
           <t>산업단지 및 다문화/공업 밀집</t>
         </is>
       </c>
+      <c r="H191" t="n">
+        <v>36.366</v>
+      </c>
+      <c r="I191" t="n">
+        <v>128.4606</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6003,6 +7153,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H192" t="n">
+        <v>36.401</v>
+      </c>
+      <c r="I192" t="n">
+        <v>128.2356</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6032,6 +7188,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H193" t="n">
+        <v>36.261</v>
+      </c>
+      <c r="I193" t="n">
+        <v>128.9106</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6061,6 +7223,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H194" t="n">
+        <v>36.401</v>
+      </c>
+      <c r="I194" t="n">
+        <v>129.1806</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6090,6 +7258,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H195" t="n">
+        <v>36.051</v>
+      </c>
+      <c r="I195" t="n">
+        <v>128.2806</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6119,6 +7293,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H196" t="n">
+        <v>36.156</v>
+      </c>
+      <c r="I196" t="n">
+        <v>128.0106</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -6148,6 +7328,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H197" t="n">
+        <v>36.156</v>
+      </c>
+      <c r="I197" t="n">
+        <v>128.0556</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -6177,6 +7363,12 @@
           <t>산업단지 및 다문화/공업 밀집</t>
         </is>
       </c>
+      <c r="H198" t="n">
+        <v>37.031</v>
+      </c>
+      <c r="I198" t="n">
+        <v>128.3706</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6206,6 +7398,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H199" t="n">
+        <v>36.611</v>
+      </c>
+      <c r="I199" t="n">
+        <v>128.5506</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6235,6 +7433,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H200" t="n">
+        <v>36.471</v>
+      </c>
+      <c r="I200" t="n">
+        <v>127.8756</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6264,6 +7468,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H201" t="n">
+        <v>37.066</v>
+      </c>
+      <c r="I201" t="n">
+        <v>128.9106</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6293,6 +7503,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H202" t="n">
+        <v>36.051</v>
+      </c>
+      <c r="I202" t="n">
+        <v>128.0556</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -6322,6 +7538,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H203" t="n">
+        <v>37.066</v>
+      </c>
+      <c r="I203" t="n">
+        <v>128.4606</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -6351,6 +7573,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H204" t="n">
+        <v>36.436</v>
+      </c>
+      <c r="I204" t="n">
+        <v>128.9106</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -6380,6 +7608,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H205" t="n">
+        <v>36.541</v>
+      </c>
+      <c r="I205" t="n">
+        <v>128.2356</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -6409,6 +7643,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H206" t="n">
+        <v>36.191</v>
+      </c>
+      <c r="I206" t="n">
+        <v>128.8206</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -6438,6 +7678,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H207" t="n">
+        <v>36.541</v>
+      </c>
+      <c r="I207" t="n">
+        <v>128.0556</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -6467,6 +7713,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H208" t="n">
+        <v>37.031</v>
+      </c>
+      <c r="I208" t="n">
+        <v>128.5506</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -6496,6 +7748,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H209" t="n">
+        <v>36.891</v>
+      </c>
+      <c r="I209" t="n">
+        <v>128.0106</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -6525,6 +7783,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H210" t="n">
+        <v>36.891</v>
+      </c>
+      <c r="I210" t="n">
+        <v>128.2356</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -6554,6 +7818,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H211" t="n">
+        <v>34.9356</v>
+      </c>
+      <c r="I211" t="n">
+        <v>127.5832</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -6583,6 +7853,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H212" t="n">
+        <v>35.4606</v>
+      </c>
+      <c r="I212" t="n">
+        <v>128.5282</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -6612,6 +7888,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H213" t="n">
+        <v>35.6006</v>
+      </c>
+      <c r="I213" t="n">
+        <v>127.7632</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -6641,6 +7923,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H214" t="n">
+        <v>35.3906</v>
+      </c>
+      <c r="I214" t="n">
+        <v>128.0332</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -6670,6 +7958,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H215" t="n">
+        <v>35.3906</v>
+      </c>
+      <c r="I215" t="n">
+        <v>127.6282</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -6699,6 +7993,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H216" t="n">
+        <v>35.3206</v>
+      </c>
+      <c r="I216" t="n">
+        <v>127.9432</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -6728,6 +8028,12 @@
           <t>대도시 중심 도심권 및 복합 상권</t>
         </is>
       </c>
+      <c r="H217" t="n">
+        <v>35.5656</v>
+      </c>
+      <c r="I217" t="n">
+        <v>127.9882</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -6757,6 +8063,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H218" t="n">
+        <v>35.7056</v>
+      </c>
+      <c r="I218" t="n">
+        <v>128.3032</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -6786,6 +8098,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H219" t="n">
+        <v>35.1106</v>
+      </c>
+      <c r="I219" t="n">
+        <v>128.1682</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -6815,6 +8133,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H220" t="n">
+        <v>35.8106</v>
+      </c>
+      <c r="I220" t="n">
+        <v>128.8432</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -6844,6 +8168,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H221" t="n">
+        <v>35.6006</v>
+      </c>
+      <c r="I221" t="n">
+        <v>127.5832</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -6873,6 +8203,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H222" t="n">
+        <v>35.0056</v>
+      </c>
+      <c r="I222" t="n">
+        <v>127.5382</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -6902,6 +8238,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H223" t="n">
+        <v>34.9706</v>
+      </c>
+      <c r="I223" t="n">
+        <v>127.5382</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -6931,6 +8273,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H224" t="n">
+        <v>35.1806</v>
+      </c>
+      <c r="I224" t="n">
+        <v>127.8982</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -6960,6 +8308,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H225" t="n">
+        <v>35.5656</v>
+      </c>
+      <c r="I225" t="n">
+        <v>128.7982</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -6989,6 +8343,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H226" t="n">
+        <v>35.7056</v>
+      </c>
+      <c r="I226" t="n">
+        <v>127.9432</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -7018,6 +8378,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H227" t="n">
+        <v>35.0056</v>
+      </c>
+      <c r="I227" t="n">
+        <v>127.5832</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -7047,6 +8413,12 @@
           <t>전원형 농어촌 및 고령 주거지</t>
         </is>
       </c>
+      <c r="H228" t="n">
+        <v>35.7056</v>
+      </c>
+      <c r="I228" t="n">
+        <v>128.3032</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7076,6 +8448,12 @@
           <t>주거 밀집 베드타운</t>
         </is>
       </c>
+      <c r="H229" t="n">
+        <v>33.2541</v>
+      </c>
+      <c r="I229" t="n">
+        <v>126.5601</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7104,6 +8482,12 @@
         <is>
           <t>주거 밀집 베드타운</t>
         </is>
+      </c>
+      <c r="H230" t="n">
+        <v>33.4996</v>
+      </c>
+      <c r="I230" t="n">
+        <v>126.5312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>